<commit_message>
Add script to remove AppImage
</commit_message>
<xml_diff>
--- a/Ubuntu-Optimize-On-Thinkpad.xlsx
+++ b/Ubuntu-Optimize-On-Thinkpad.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
   <si>
     <t xml:space="preserve">STT</t>
   </si>
@@ -185,6 +185,24 @@
   </si>
   <si>
     <t xml:space="preserve">Ép BIOS chỉ tập trung đọc phân vùng ổ cứng NVMe chứa Ubuntu, tăng tốc độ POST phần cứng lên mức tối đa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tự động hóa Power Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/etc/udev/rules.d/99-power-profile.rules
+/usr/local/bin/auto-power-profile.sh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cắm sạc $\rightarrow$ balanced
+Rút sạc $\rightarrow$ power-saver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cắm sạc $\rightarrow$ performance
+Rút sạc $\rightarrow$ power-saver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giải phóng 100% sức mạnh CPU i7 khi làm việc tại bàn; tự động ép máy chạy mát và tiết kiệm pin khi di chuyển.</t>
   </si>
 </sst>
 </file>
@@ -195,7 +213,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="d\.m"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -219,10 +237,25 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b val="true"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -275,21 +308,41 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -482,236 +535,257 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="39.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="57.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="64.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="39.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="57.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="64.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="99"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="n">
         <v>46023</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+    <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="n">
         <v>46024</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="n">
         <v>46055</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
         <v>46083</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
         <v>46025</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
         <v>46056</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
         <v>46026</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
         <v>46027</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="n">
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
         <v>46028</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
         <v>46059</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="7" t="s">
         <v>51</v>
       </c>
     </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>